<commit_message>
Atualiza populacao e renda para o Censo 2022 (IBGE, setores censitarios)
</commit_message>
<xml_diff>
--- a/output/indicadores_gtfs.xlsx
+++ b/output/indicadores_gtfs.xlsx
@@ -15,13 +15,14 @@
     <sheet name="Velocidade linhas" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Cobertura" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Cobertura empregos" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Sem servico freq" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Censo 2022 x 2010" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Sem servico freq" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1260" uniqueCount="1260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1264" uniqueCount="1264">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -3764,6 +3765,9 @@
     <t xml:space="preserve">populacao</t>
   </si>
   <si>
+    <t xml:space="preserve">renda_media_resp</t>
+  </si>
+  <si>
     <t xml:space="preserve">pct_qualquer</t>
   </si>
   <si>
@@ -3795,6 +3799,15 @@
   </si>
   <si>
     <t xml:space="preserve">pct_empregos_frequente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Censo 2022 (IBGE, usado na análise)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Censo 2010 (IPEA)</t>
   </si>
   <si>
     <t xml:space="preserve">quintil</t>
@@ -4333,56 +4346,125 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
+    <col min="1" max="1" width="36.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="9.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="12.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="13.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="18.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>1259</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1248</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1249</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>1260</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2422743</v>
+      </c>
+      <c r="C2" t="n">
+        <v>99.25</v>
+      </c>
+      <c r="D2" t="n">
+        <v>76.84</v>
+      </c>
+      <c r="E2" t="n">
+        <v>46.83</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>1261</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2418518</v>
+      </c>
+      <c r="C3" t="n">
+        <v>99.66</v>
+      </c>
+      <c r="D3" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>48.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
     <col min="1" max="1" width="20.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="16.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1258</v>
+        <v>1262</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1259</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="B2" t="n">
-        <v>130746.7</v>
+        <v>137513.39</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="B3" t="n">
-        <v>107954.45</v>
+        <v>105488.48</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="B4" t="n">
-        <v>94309.01</v>
+        <v>132925.22</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="B5" t="n">
-        <v>103056.01</v>
+        <v>107475.36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="B6" t="n">
-        <v>59730.99</v>
+        <v>77679.69</v>
       </c>
     </row>
   </sheetData>
@@ -31513,9 +31595,10 @@
   <cols>
     <col min="1" max="1" width="20.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="9.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="12.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="13.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="18.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="16.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="12.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="13.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="18.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -31534,107 +31617,126 @@
       <c r="E1" s="1" t="s">
         <v>1249</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>1250</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1250</v>
+        <v>1251</v>
       </c>
       <c r="B2" t="n">
-        <v>2418518</v>
-      </c>
-      <c r="C2" t="n">
-        <v>99.66</v>
-      </c>
+        <v>2422743</v>
+      </c>
+      <c r="C2"/>
       <c r="D2" t="n">
-        <v>79.5</v>
+        <v>99.25</v>
       </c>
       <c r="E2" t="n">
-        <v>48.8</v>
+        <v>76.84</v>
+      </c>
+      <c r="F2" t="n">
+        <v>46.83</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="B3" t="n">
-        <v>483277</v>
+        <v>484530.85</v>
       </c>
       <c r="C3" t="n">
-        <v>99.17</v>
+        <v>1280.48</v>
       </c>
       <c r="D3" t="n">
-        <v>72.95</v>
+        <v>99.13</v>
       </c>
       <c r="E3" t="n">
-        <v>28.33</v>
+        <v>71.62</v>
+      </c>
+      <c r="F3" t="n">
+        <v>29.76</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="B4" t="n">
-        <v>484774</v>
+        <v>483788.77</v>
       </c>
       <c r="C4" t="n">
-        <v>99.8</v>
+        <v>1546.83</v>
       </c>
       <c r="D4" t="n">
-        <v>77.73</v>
+        <v>99.33</v>
       </c>
       <c r="E4" t="n">
-        <v>39.98</v>
+        <v>78.2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>38.69</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="B5" t="n">
-        <v>482215</v>
+        <v>485414.56</v>
       </c>
       <c r="C5" t="n">
-        <v>99.81</v>
+        <v>1939.66</v>
       </c>
       <c r="D5" t="n">
-        <v>80.44</v>
+        <v>99.28</v>
       </c>
       <c r="E5" t="n">
-        <v>48.23</v>
+        <v>72.62</v>
+      </c>
+      <c r="F5" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="B6" t="n">
-        <v>484097</v>
+        <v>483812.25</v>
       </c>
       <c r="C6" t="n">
-        <v>99.75</v>
+        <v>2756.55</v>
       </c>
       <c r="D6" t="n">
-        <v>78.71</v>
+        <v>99.36</v>
       </c>
       <c r="E6" t="n">
-        <v>56.51</v>
+        <v>77.79</v>
+      </c>
+      <c r="F6" t="n">
+        <v>54.18</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="B7" t="n">
-        <v>484155</v>
+        <v>485196.58</v>
       </c>
       <c r="C7" t="n">
-        <v>99.75</v>
+        <v>7470.97</v>
       </c>
       <c r="D7" t="n">
-        <v>87.66</v>
+        <v>99.19</v>
       </c>
       <c r="E7" t="n">
-        <v>70.91</v>
+        <v>83.99</v>
+      </c>
+      <c r="F7" t="n">
+        <v>67.52</v>
       </c>
     </row>
   </sheetData>
@@ -31654,10 +31756,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1257</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="2">

</xml_diff>